<commit_message>
feat: separate dedicated /talabalar and /xodimlar pages with URL routing and enriched teacher records
</commit_message>
<xml_diff>
--- a/hisobotlar/Barcha xodimlar royxati.xlsx
+++ b/hisobotlar/Barcha xodimlar royxati.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -470,13 +470,16 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -514,40 +517,55 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Pedagogik toifasi</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>Telefon raqami</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Tug'ilgan sanasi</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Pasport seriya va raqami</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>JSHSHIR (PINFL)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>INN (STIR)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Plastik karta raqami</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Tamomlagan OTM / Ta'lim muassasasi</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Diplom bo'yicha mutaxassisligi</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Ishga kirgan buyruq sanasi</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Holati</t>
         </is>
@@ -577,42 +595,49 @@
           <t>Rahbariyat</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>+998 94 336 66 44</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>12.11.1983</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>AD 5424248</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>31211832710036</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>9860080311468542</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Mirzo Ulug'bek nomidagi O'zbekiston Milliy universiteti</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Ijtimoiy tizimlar va jarayonlarning axborot psixalogik xavfsizligi</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -642,34 +667,41 @@
           <t>Rahbariyat</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>+998 97 587 46 57</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>10.08.1993</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>AD 8142516</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>31008932640046</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr"/>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
+          <t>9860080311717658</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr"/>
+      <c r="N4" s="4" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -699,34 +731,41 @@
           <t>Ma'muriy</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>+998 88 617 68 32</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>12.07.2005</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>AD 1640374</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>51207055730023</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
+          <t>9860080311682803</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -756,34 +795,41 @@
           <t>Xo'jalik</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>+998 91 221 31 64</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>28.05.1962</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>AB 0313713</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>32805622730035</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr"/>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
+          <t>9860080311417465</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -813,34 +859,41 @@
           <t>Xo'jalik</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>+998 90 670 30 78</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>30.04.1978</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>AC 0062427</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>43004787890011</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
+          <t>9860080311516175</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -870,34 +923,41 @@
           <t>Tibbiy xizmat</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>+998 91 643 10 05</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>11.11.1989</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>AA 9203328</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>41111892560099</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
+          <t>9860080311452975</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -927,34 +987,37 @@
           <t>Ma'muriy</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>+998 99 264 81 86</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>15.01.1981</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>AD 5429893</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>31501815560016</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
-      <c r="K9" s="4" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr"/>
+      <c r="O9" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="P9" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -984,34 +1047,41 @@
           <t>Ma'muriy</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>+998 88 589 20 26</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>26.03.2000</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>AB 6194841</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>62603005590051</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
+          <t>9860080311950358</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1041,42 +1111,53 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>+998 94 485 66 86</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>11.12.1986</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>AD 6387297</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>31112862640255</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>531026980</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>9860080311188025</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
         <is>
           <t>Toshkent Pediatriya Tibbiyot instituti</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>Oliy hamshiralik ishi</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1106,42 +1187,53 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>+998 91 470 39 64</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>11.02.1988</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>AE 4760879</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>31102882560109</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>521992768</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>9860080311251534</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiyasi</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="N12" s="4" t="inlineStr">
         <is>
           <t>Oliy ma'lumotli hamshira</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1171,42 +1263,53 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>+998 90 864 21 55</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>05.09.1957</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>AB 1389306</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>40509572560045</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>535156144</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>9860080311146577</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>Samarqand davlat meditsina universiteti</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>Davolash</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="P13" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1236,42 +1339,49 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>+998 99 775 40 49</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>09.05.1988</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>AD 3879994</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>40905885590016</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>9860080311922456</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiyasi</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="N14" s="4" t="inlineStr">
         <is>
           <t>Oliy ma'lumotli hamshira</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1301,42 +1411,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>+998 91 961 03 04</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>20.09.1987</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>AB 6572306</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>32009872640056</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
         <is>
           <t>Toshkent farmatsevtika instituti</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>Biotexnalogiya</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1366,42 +1479,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>+998 90 313 05 00</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>15.01.1998</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>AE 3698603</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>41501985680018</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
         <is>
           <t>O'zbekiston jahon tillari universiteti</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="N16" s="4" t="inlineStr">
         <is>
           <t>Ingliz tili va adabiyot o'qituvchisi</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1431,42 +1547,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>+998 88 260 86 68</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>07.12.1989</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>AE 2829988</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>40712892560095</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr">
         <is>
           <t>Mirzo Ulug'bek nomidagi O'zbekiston Milliy universiteti</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>Biokimyo</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="O17" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="P17" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1496,42 +1615,53 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>+998 97 381 34 33</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>12.01.1987</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>AD 0594238</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>31201872730017</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>508274139</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>9860080311919635</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
         <is>
           <t>Mirzo Ulug'bek nomidagi O'zbekiston Milliy universiteti</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="N18" s="4" t="inlineStr">
         <is>
           <t>Falsafa</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1561,42 +1691,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>+998 91 462 66 48</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>16.10.1988</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>AD 6227655</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>41610882560070</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="K19" s="3" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiyasi</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>Oliy hamshiralik ishi</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="P19" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1626,42 +1759,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>+998 77 023 01 46</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>03.04.2001</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>AC 1298495</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>60304017890020</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="K20" s="3" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiyasi</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Oliy hamshiralik ishi</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1691,42 +1827,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>+998 91 810 06 14</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>14.06.1999</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>AB 6147908</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>41406995590053</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="K21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiysi</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>Oliy ma'lumotli hamshira</t>
         </is>
       </c>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="O21" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="P21" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1756,42 +1895,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>+998 88 589 29 21</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>22.04.1992</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>AE3796962</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>42204922560080</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiysi</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="N22" s="4" t="inlineStr">
         <is>
           <t>Oliy ma'lumotli hamshira</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1821,42 +1963,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>+998 88 564 14 41</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>14.07.1985</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>AB 7576700</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>41407852560095</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr">
         <is>
           <t>Toshkent farmatsevtika instituti</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>Farmatsiya</t>
         </is>
       </c>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="O23" s="3" t="inlineStr">
         <is>
           <t>28.08.2026</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="P23" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1886,42 +2031,49 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>+998 91 213 93 59</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>28.08.1981</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>AA 6393123</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>42808815590011</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="K24" s="3" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>9860080311533196</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
         <is>
           <t>Toshkent Pediateriya tibbiyot instituti</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="N24" s="4" t="inlineStr">
         <is>
           <t>Oliy hamshiralik ishi</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -1951,42 +2103,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>+998 90 517 05 15</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>11.11.1981</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>AD 5571124</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>41111812640038</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>Samarqand davlat tibbiyot instituti</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>Oliy ma'lumotli hamshira</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="O25" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="P25" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2016,42 +2171,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>+998 97 380 86 17</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>18.06.1976</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>AB 4848015</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>41806765590023</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Shahrisabz tibbiyot bilim yurti</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="N26" s="4" t="inlineStr">
         <is>
           <t>Tibbiy hamshira</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="P26" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2081,42 +2239,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>+998 88 854 87 97</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>18.04.1989</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>AD 8366544</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>31804892560060</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr">
         <is>
           <t>Samarqand davlat tibbiyot instituti</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>Pediateriya ishi bo'yicha umumiy amaliyot vrach pediateri</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr">
+      <c r="O27" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="P27" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2146,42 +2307,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>+998 97 631 81 87</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>27.11.1987</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>AD 1713547</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>42711872560032</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr">
         <is>
           <t>Shahrisabz tibiyot kolleji</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="N28" s="4" t="inlineStr">
         <is>
           <t>Umumiy amaliyot hamshirasi</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="O28" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2211,42 +2375,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>+998 91 636 35 98</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>27.11.1990</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>AB 9132346</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>42711902560072</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="K29" s="3" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr">
         <is>
           <t>ILM-U ZIYO BIZNES IBBIYOT TEXNIKUMI</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>Hamshiralik ishi</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="O29" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="P29" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2276,42 +2443,45 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>+998 90 186 05 33</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>04.07.1985</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>AB 6655981</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>30407852530018</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr">
         <is>
           <t>Toshkent tibbiyot akademiyasi</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="N30" s="4" t="inlineStr">
         <is>
           <t>Umumiy amaliyot vrachi</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2341,42 +2511,53 @@
           <t>Pedagog</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>+998 90 129 90 08</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>03.09.1995</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>AE 2643207</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>40309952640064</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>598582343</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>9860080311393286</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
         <is>
           <t>ALFRAGANUS UNIVERSITY</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>Umumiy stomatolog shifokori</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="O31" s="3" t="inlineStr">
         <is>
           <t>28.09.2026</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="P31" s="3" t="inlineStr">
         <is>
           <t>Faol</t>
         </is>
@@ -2384,7 +2565,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>